<commit_message>
Import rules: field mapping, scan-event grouping, arrival date, conflicts
- docs/import-rules.md: tracking code = scan order number (kept as text);
  configurable mappings with a fixed Shopee SHPE filter; rule
  scan-events-to-parcels/v1 (collapse repeat scans, earliest arrived scan
  time as arrival date, name/phone conflicts and missing arrival flagged for
  staff, existing parcels never overwritten); verified real-export counts.
- test/fixtures: extended scan-record-mixed (conflicts, missing arrival,
  earliest-arrival, leading-zero and letter codes, two split rows) in all
  four formats; header fixtures for missing/duplicated columns.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test/fixtures/scan-record-mixed.xlsx
+++ b/test/fixtures/scan-record-mixed.xlsx
@@ -8,7 +8,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="134">
   <si>
     <t xml:space="preserve">scan order number</t>
   </si>
@@ -109,6 +109,9 @@
     <t xml:space="preserve">Test Hub</t>
   </si>
   <si>
+    <t xml:space="preserve">2026-10-10 09:00:00</t>
+  </si>
+  <si>
     <t xml:space="preserve">Shopee SHPE</t>
   </si>
   <si>
@@ -190,6 +193,12 @@
     <t xml:space="preserve">012345670</t>
   </si>
   <si>
+    <t xml:space="preserve">2026-10-10 07:30:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-09 23:50:00</t>
+  </si>
+  <si>
     <t xml:space="preserve">10000000000006</t>
   </si>
   <si>
@@ -223,7 +232,7 @@
     <t xml:space="preserve">10000000000008</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-10-10 08:08:00</t>
+    <t xml:space="preserve">2026-10-10 07:08:00</t>
   </si>
   <si>
     <t xml:space="preserve">Siem Reap Province SRP-01</t>
@@ -244,6 +253,12 @@
     <t xml:space="preserve">2026-10-10 08:09:00</t>
   </si>
   <si>
+    <t xml:space="preserve">X000000002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-10 08:09:30</t>
+  </si>
+  <si>
     <t xml:space="preserve">10000000000009</t>
   </si>
   <si>
@@ -311,6 +326,90 @@
   </si>
   <si>
     <t xml:space="preserve">855123456713</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10000000000014</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-10 08:15:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test Customer O</t>
+  </si>
+  <si>
+    <t xml:space="preserve">855123456714</t>
+  </si>
+  <si>
+    <t xml:space="preserve">855123456799</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10000000000015</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-10 08:16:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test Customer P</t>
+  </si>
+  <si>
+    <t xml:space="preserve">855123456715</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-10 07:16:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test Customer R</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10000000000016</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-10 08:17:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> test customer q </t>
+  </si>
+  <si>
+    <t xml:space="preserve">855-0123456716</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-10 07:17:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test Customer Q</t>
+  </si>
+  <si>
+    <t xml:space="preserve">855123456716</t>
+  </si>
+  <si>
+    <t xml:space="preserve">00000000000017</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-10 08:18:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test Customer S</t>
+  </si>
+  <si>
+    <t xml:space="preserve">855123456717</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Arrived </t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-10 07:18:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S000000018</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-10 07:19:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test Customer T</t>
+  </si>
+  <si>
+    <t xml:space="preserve">855123456718</t>
   </si>
 </sst>
 </file>
@@ -445,10 +544,10 @@
         <v>30</v>
       </c>
       <c r="I2" t="s" s="1">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="J2" t="s" s="1">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="K2" t="s" s="1">
         <v>31</v>
@@ -469,22 +568,22 @@
         <v>0</v>
       </c>
       <c r="Q2" t="s" s="1">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="R2" t="s" s="1">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="S2" t="s" s="1">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="T2" t="s" s="1">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="Y2" t="s" s="1">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="Z2" t="s" s="1">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="3">
@@ -495,10 +594,10 @@
         <v>27</v>
       </c>
       <c r="C3" t="s" s="1">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D3" t="s" s="1">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E3" t="s" s="1">
         <v>30</v>
@@ -513,10 +612,10 @@
         <v>30</v>
       </c>
       <c r="I3" t="s" s="1">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="J3" t="s" s="1">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="K3" t="s" s="1">
         <v>31</v>
@@ -537,27 +636,27 @@
         <v>0</v>
       </c>
       <c r="Q3" t="s" s="1">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="R3" t="s" s="1">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="S3" t="s" s="1">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="T3" t="s" s="1">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="Y3" t="s" s="1">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="Z3" t="s" s="1">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="1">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B4" t="s" s="1">
         <v>27</v>
@@ -566,7 +665,7 @@
         <v>28</v>
       </c>
       <c r="D4" t="s" s="1">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E4" t="s" s="1">
         <v>30</v>
@@ -581,10 +680,10 @@
         <v>30</v>
       </c>
       <c r="I4" t="s" s="1">
-        <v>42</v>
+        <v>33</v>
       </c>
       <c r="J4" t="s" s="1">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="K4" t="s" s="1">
         <v>31</v>
@@ -605,27 +704,27 @@
         <v>0</v>
       </c>
       <c r="Q4" t="s" s="1">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="R4" t="s" s="1">
+        <v>45</v>
+      </c>
+      <c r="S4" t="s" s="1">
+        <v>46</v>
+      </c>
+      <c r="T4" t="s" s="1">
+        <v>38</v>
+      </c>
+      <c r="Y4" t="s" s="1">
         <v>44</v>
       </c>
-      <c r="S4" t="s" s="1">
-        <v>45</v>
-      </c>
-      <c r="T4" t="s" s="1">
-        <v>37</v>
-      </c>
-      <c r="Y4" t="s" s="1">
-        <v>43</v>
-      </c>
       <c r="Z4" t="s" s="1">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="1">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B5" t="s" s="1">
         <v>27</v>
@@ -634,7 +733,7 @@
         <v>28</v>
       </c>
       <c r="D5" t="s" s="1">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E5" t="s" s="1">
         <v>30</v>
@@ -649,10 +748,10 @@
         <v>30</v>
       </c>
       <c r="I5" t="s" s="1">
-        <v>47</v>
+        <v>33</v>
       </c>
       <c r="J5" t="s" s="1">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="K5" t="s" s="1">
         <v>31</v>
@@ -673,27 +772,27 @@
         <v>0</v>
       </c>
       <c r="Q5" t="s" s="1">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="R5" t="s" s="1">
+        <v>50</v>
+      </c>
+      <c r="S5" t="s" s="1">
+        <v>51</v>
+      </c>
+      <c r="T5" t="s" s="1">
+        <v>38</v>
+      </c>
+      <c r="Y5" t="s" s="1">
         <v>49</v>
       </c>
-      <c r="S5" t="s" s="1">
-        <v>50</v>
-      </c>
-      <c r="T5" t="s" s="1">
-        <v>37</v>
-      </c>
-      <c r="Y5" t="s" s="1">
-        <v>48</v>
-      </c>
       <c r="Z5" t="s" s="1">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s" s="1">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B6" t="s" s="1">
         <v>27</v>
@@ -702,7 +801,7 @@
         <v>28</v>
       </c>
       <c r="D6" t="s" s="1">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="E6" t="s" s="1">
         <v>30</v>
@@ -717,10 +816,10 @@
         <v>30</v>
       </c>
       <c r="I6" t="s" s="1">
-        <v>52</v>
+        <v>33</v>
       </c>
       <c r="J6" t="s" s="1">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="K6" t="s" s="1">
         <v>31</v>
@@ -741,27 +840,27 @@
         <v>0</v>
       </c>
       <c r="Q6" t="s" s="1">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="R6" t="s" s="1">
+        <v>55</v>
+      </c>
+      <c r="S6" t="s" s="1">
+        <v>56</v>
+      </c>
+      <c r="T6" t="s" s="1">
+        <v>38</v>
+      </c>
+      <c r="Y6" t="s" s="1">
         <v>54</v>
       </c>
-      <c r="S6" t="s" s="1">
-        <v>55</v>
-      </c>
-      <c r="T6" t="s" s="1">
-        <v>37</v>
-      </c>
-      <c r="Y6" t="s" s="1">
-        <v>53</v>
-      </c>
       <c r="Z6" t="s" s="1">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s" s="1">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B7" t="s" s="1">
         <v>27</v>
@@ -770,7 +869,7 @@
         <v>28</v>
       </c>
       <c r="D7" t="s" s="1">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E7" t="s" s="1">
         <v>30</v>
@@ -785,10 +884,10 @@
         <v>30</v>
       </c>
       <c r="I7" t="s" s="1">
-        <v>57</v>
+        <v>33</v>
       </c>
       <c r="J7" t="s" s="1">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="K7" t="s" s="1">
         <v>31</v>
@@ -809,33 +908,33 @@
         <v>0</v>
       </c>
       <c r="Q7" t="s" s="1">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="R7" t="s" s="1">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="S7" t="s" s="1">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="T7" t="s" s="1">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="Y7" t="s" s="1">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="Z7" t="s" s="1">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s" s="1">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="B8" t="s" s="1">
         <v>27</v>
       </c>
       <c r="C8" t="s" s="1">
-        <v>28</v>
+        <v>40</v>
       </c>
       <c r="D8" t="s" s="1">
         <v>61</v>
@@ -853,10 +952,10 @@
         <v>30</v>
       </c>
       <c r="I8" t="s" s="1">
-        <v>61</v>
+        <v>33</v>
       </c>
       <c r="J8" t="s" s="1">
-        <v>62</v>
+        <v>34</v>
       </c>
       <c r="K8" t="s" s="1">
         <v>31</v>
@@ -877,36 +976,36 @@
         <v>0</v>
       </c>
       <c r="Q8" t="s" s="1">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="R8" t="s" s="1">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="S8" t="s" s="1">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="T8" t="s" s="1">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="Y8" t="s" s="1">
-        <v>62</v>
+        <v>34</v>
       </c>
       <c r="Z8" t="s" s="1">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s" s="1">
-        <v>65</v>
+        <v>57</v>
       </c>
       <c r="B9" t="s" s="1">
         <v>27</v>
       </c>
       <c r="C9" t="s" s="1">
-        <v>28</v>
+        <v>40</v>
       </c>
       <c r="D9" t="s" s="1">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="E9" t="s" s="1">
         <v>30</v>
@@ -921,10 +1020,10 @@
         <v>30</v>
       </c>
       <c r="I9" t="s" s="1">
-        <v>66</v>
+        <v>33</v>
       </c>
       <c r="J9" t="s" s="1">
-        <v>67</v>
+        <v>34</v>
       </c>
       <c r="K9" t="s" s="1">
         <v>31</v>
@@ -945,27 +1044,27 @@
         <v>0</v>
       </c>
       <c r="Q9" t="s" s="1">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="R9" t="s" s="1">
-        <v>68</v>
+        <v>59</v>
       </c>
       <c r="S9" t="s" s="1">
-        <v>69</v>
+        <v>60</v>
       </c>
       <c r="T9" t="s" s="1">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="Y9" t="s" s="1">
-        <v>67</v>
+        <v>34</v>
       </c>
       <c r="Z9" t="s" s="1">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s" s="1">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="B10" t="s" s="1">
         <v>27</v>
@@ -974,7 +1073,7 @@
         <v>28</v>
       </c>
       <c r="D10" t="s" s="1">
-        <v>71</v>
+        <v>64</v>
       </c>
       <c r="E10" t="s" s="1">
         <v>30</v>
@@ -989,10 +1088,10 @@
         <v>30</v>
       </c>
       <c r="I10" t="s" s="1">
-        <v>71</v>
+        <v>33</v>
       </c>
       <c r="J10" t="s" s="1">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="K10" t="s" s="1">
         <v>31</v>
@@ -1013,36 +1112,36 @@
         <v>0</v>
       </c>
       <c r="Q10" t="s" s="1">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="R10" t="s" s="1">
-        <v>73</v>
+        <v>66</v>
       </c>
       <c r="S10" t="s" s="1">
-        <v>74</v>
+        <v>67</v>
       </c>
       <c r="T10" t="s" s="1">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="Y10" t="s" s="1">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="Z10" t="s" s="1">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s" s="1">
-        <v>75</v>
+        <v>68</v>
       </c>
       <c r="B11" t="s" s="1">
         <v>27</v>
       </c>
       <c r="C11" t="s" s="1">
-        <v>76</v>
+        <v>28</v>
       </c>
       <c r="D11" t="s" s="1">
-        <v>77</v>
+        <v>69</v>
       </c>
       <c r="E11" t="s" s="1">
         <v>30</v>
@@ -1050,28 +1149,67 @@
       <c r="F11" t="s" s="1">
         <v>31</v>
       </c>
+      <c r="G11" t="s" s="1">
+        <v>32</v>
+      </c>
       <c r="H11" t="s" s="1">
         <v>30</v>
       </c>
       <c r="I11" t="s" s="1">
-        <v>77</v>
+        <v>33</v>
+      </c>
+      <c r="J11" t="s" s="1">
+        <v>70</v>
+      </c>
+      <c r="K11" t="s" s="1">
+        <v>31</v>
+      </c>
+      <c r="L11">
+        <v>1</v>
       </c>
       <c r="M11">
         <v>0.5</v>
+      </c>
+      <c r="N11">
+        <v>0.5</v>
+      </c>
+      <c r="O11">
+        <v>0</v>
+      </c>
+      <c r="P11">
+        <v>0</v>
+      </c>
+      <c r="Q11" t="s" s="1">
+        <v>35</v>
+      </c>
+      <c r="R11" t="s" s="1">
+        <v>71</v>
+      </c>
+      <c r="S11" t="s" s="1">
+        <v>72</v>
+      </c>
+      <c r="T11" t="s" s="1">
+        <v>38</v>
+      </c>
+      <c r="Y11" t="s" s="1">
+        <v>70</v>
+      </c>
+      <c r="Z11" t="s" s="1">
+        <v>39</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s" s="1">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="B12" t="s" s="1">
         <v>27</v>
       </c>
       <c r="C12" t="s" s="1">
-        <v>28</v>
+        <v>40</v>
       </c>
       <c r="D12" t="s" s="1">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="E12" t="s" s="1">
         <v>30</v>
@@ -1086,10 +1224,10 @@
         <v>30</v>
       </c>
       <c r="I12" t="s" s="1">
-        <v>79</v>
+        <v>33</v>
       </c>
       <c r="J12" t="s" s="1">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="K12" t="s" s="1">
         <v>31</v>
@@ -1110,36 +1248,36 @@
         <v>0</v>
       </c>
       <c r="Q12" t="s" s="1">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="R12" t="s" s="1">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="S12" t="s" s="1">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="T12" t="s" s="1">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="Y12" t="s" s="1">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="Z12" t="s" s="1">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s" s="1">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="B13" t="s" s="1">
         <v>27</v>
       </c>
       <c r="C13" t="s" s="1">
-        <v>28</v>
+        <v>79</v>
       </c>
       <c r="D13" t="s" s="1">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="E13" t="s" s="1">
         <v>30</v>
@@ -1147,67 +1285,28 @@
       <c r="F13" t="s" s="1">
         <v>31</v>
       </c>
-      <c r="G13" t="s" s="1">
-        <v>32</v>
-      </c>
       <c r="H13" t="s" s="1">
         <v>30</v>
       </c>
       <c r="I13" t="s" s="1">
-        <v>84</v>
-      </c>
-      <c r="J13" t="s" s="1">
-        <v>85</v>
-      </c>
-      <c r="K13" t="s" s="1">
-        <v>31</v>
-      </c>
-      <c r="L13">
-        <v>1</v>
+        <v>33</v>
       </c>
       <c r="M13">
         <v>0.5</v>
-      </c>
-      <c r="N13">
-        <v>0.5</v>
-      </c>
-      <c r="O13">
-        <v>0</v>
-      </c>
-      <c r="P13">
-        <v>0</v>
-      </c>
-      <c r="Q13" t="s" s="1">
-        <v>34</v>
-      </c>
-      <c r="R13" t="s" s="1">
-        <v>86</v>
-      </c>
-      <c r="S13" t="s" s="1">
-        <v>87</v>
-      </c>
-      <c r="T13" t="s" s="1">
-        <v>37</v>
-      </c>
-      <c r="Y13" t="s" s="1">
-        <v>85</v>
-      </c>
-      <c r="Z13" t="s" s="1">
-        <v>38</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s" s="1">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="B14" t="s" s="1">
         <v>27</v>
       </c>
       <c r="C14" t="s" s="1">
-        <v>28</v>
+        <v>79</v>
       </c>
       <c r="D14" t="s" s="1">
-        <v>89</v>
+        <v>82</v>
       </c>
       <c r="E14" t="s" s="1">
         <v>30</v>
@@ -1215,58 +1314,19 @@
       <c r="F14" t="s" s="1">
         <v>31</v>
       </c>
-      <c r="G14" t="s" s="1">
-        <v>32</v>
-      </c>
       <c r="H14" t="s" s="1">
         <v>30</v>
       </c>
       <c r="I14" t="s" s="1">
-        <v>89</v>
-      </c>
-      <c r="J14" t="s" s="1">
-        <v>90</v>
-      </c>
-      <c r="K14" t="s" s="1">
-        <v>31</v>
-      </c>
-      <c r="L14">
-        <v>1</v>
+        <v>33</v>
       </c>
       <c r="M14">
         <v>0.5</v>
-      </c>
-      <c r="N14">
-        <v>0.5</v>
-      </c>
-      <c r="O14">
-        <v>0</v>
-      </c>
-      <c r="P14">
-        <v>0</v>
-      </c>
-      <c r="Q14" t="s" s="1">
-        <v>34</v>
-      </c>
-      <c r="R14" t="s" s="1">
-        <v>91</v>
-      </c>
-      <c r="S14" t="s" s="1">
-        <v>92</v>
-      </c>
-      <c r="T14" t="s" s="1">
-        <v>37</v>
-      </c>
-      <c r="Y14" t="s" s="1">
-        <v>90</v>
-      </c>
-      <c r="Z14" t="s" s="1">
-        <v>38</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s" s="1">
-        <v>93</v>
+        <v>83</v>
       </c>
       <c r="B15" t="s" s="1">
         <v>27</v>
@@ -1275,7 +1335,7 @@
         <v>28</v>
       </c>
       <c r="D15" t="s" s="1">
-        <v>94</v>
+        <v>84</v>
       </c>
       <c r="E15" t="s" s="1">
         <v>30</v>
@@ -1290,10 +1350,10 @@
         <v>30</v>
       </c>
       <c r="I15" t="s" s="1">
-        <v>94</v>
+        <v>33</v>
       </c>
       <c r="J15" t="s" s="1">
-        <v>95</v>
+        <v>85</v>
       </c>
       <c r="K15" t="s" s="1">
         <v>31</v>
@@ -1314,27 +1374,27 @@
         <v>0</v>
       </c>
       <c r="Q15" t="s" s="1">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="R15" t="s" s="1">
-        <v>96</v>
+        <v>86</v>
       </c>
       <c r="S15" t="s" s="1">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="T15" t="s" s="1">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="Y15" t="s" s="1">
-        <v>95</v>
+        <v>85</v>
       </c>
       <c r="Z15" t="s" s="1">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s" s="1">
-        <v>41</v>
+        <v>88</v>
       </c>
       <c r="B16" t="s" s="1">
         <v>27</v>
@@ -1343,61 +1403,877 @@
         <v>28</v>
       </c>
       <c r="D16" t="s" s="1">
+        <v>89</v>
+      </c>
+      <c r="E16" t="s" s="1">
+        <v>30</v>
+      </c>
+      <c r="F16" t="s" s="1">
+        <v>31</v>
+      </c>
+      <c r="G16" t="s" s="1">
+        <v>32</v>
+      </c>
+      <c r="H16" t="s" s="1">
+        <v>30</v>
+      </c>
+      <c r="I16" t="s" s="1">
+        <v>33</v>
+      </c>
+      <c r="J16" t="s" s="1">
+        <v>90</v>
+      </c>
+      <c r="K16" t="s" s="1">
+        <v>31</v>
+      </c>
+      <c r="L16">
+        <v>1</v>
+      </c>
+      <c r="M16">
+        <v>0.5</v>
+      </c>
+      <c r="N16">
+        <v>0.5</v>
+      </c>
+      <c r="O16">
+        <v>0</v>
+      </c>
+      <c r="P16">
+        <v>0</v>
+      </c>
+      <c r="Q16" t="s" s="1">
+        <v>35</v>
+      </c>
+      <c r="R16" t="s" s="1">
+        <v>91</v>
+      </c>
+      <c r="S16" t="s" s="1">
+        <v>92</v>
+      </c>
+      <c r="T16" t="s" s="1">
+        <v>38</v>
+      </c>
+      <c r="Y16" t="s" s="1">
+        <v>90</v>
+      </c>
+      <c r="Z16" t="s" s="1">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s" s="1">
+        <v>93</v>
+      </c>
+      <c r="B17" t="s" s="1">
+        <v>27</v>
+      </c>
+      <c r="C17" t="s" s="1">
+        <v>28</v>
+      </c>
+      <c r="D17" t="s" s="1">
+        <v>94</v>
+      </c>
+      <c r="E17" t="s" s="1">
+        <v>30</v>
+      </c>
+      <c r="F17" t="s" s="1">
+        <v>31</v>
+      </c>
+      <c r="G17" t="s" s="1">
+        <v>32</v>
+      </c>
+      <c r="H17" t="s" s="1">
+        <v>30</v>
+      </c>
+      <c r="I17" t="s" s="1">
+        <v>33</v>
+      </c>
+      <c r="J17" t="s" s="1">
+        <v>95</v>
+      </c>
+      <c r="K17" t="s" s="1">
+        <v>31</v>
+      </c>
+      <c r="L17">
+        <v>1</v>
+      </c>
+      <c r="M17">
+        <v>0.5</v>
+      </c>
+      <c r="N17">
+        <v>0.5</v>
+      </c>
+      <c r="O17">
+        <v>0</v>
+      </c>
+      <c r="P17">
+        <v>0</v>
+      </c>
+      <c r="Q17" t="s" s="1">
+        <v>35</v>
+      </c>
+      <c r="R17" t="s" s="1">
+        <v>96</v>
+      </c>
+      <c r="S17" t="s" s="1">
+        <v>97</v>
+      </c>
+      <c r="T17" t="s" s="1">
+        <v>38</v>
+      </c>
+      <c r="Y17" t="s" s="1">
+        <v>95</v>
+      </c>
+      <c r="Z17" t="s" s="1">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s" s="1">
         <v>98</v>
       </c>
-      <c r="E16" t="s" s="1">
-        <v>30</v>
-      </c>
-      <c r="F16" t="s" s="1">
-        <v>31</v>
-      </c>
-      <c r="G16" t="s" s="1">
-        <v>32</v>
-      </c>
-      <c r="H16" t="s" s="1">
-        <v>30</v>
-      </c>
-      <c r="I16" t="s" s="1">
-        <v>98</v>
-      </c>
-      <c r="J16" t="s" s="1">
-        <v>62</v>
-      </c>
-      <c r="K16" t="s" s="1">
-        <v>31</v>
-      </c>
-      <c r="L16">
-        <v>1</v>
-      </c>
-      <c r="M16">
-        <v>0.5</v>
-      </c>
-      <c r="N16">
-        <v>0.5</v>
-      </c>
-      <c r="O16">
-        <v>0</v>
-      </c>
-      <c r="P16">
-        <v>0</v>
-      </c>
-      <c r="Q16" t="s" s="1">
-        <v>34</v>
-      </c>
-      <c r="R16" t="s" s="1">
+      <c r="B18" t="s" s="1">
+        <v>27</v>
+      </c>
+      <c r="C18" t="s" s="1">
+        <v>28</v>
+      </c>
+      <c r="D18" t="s" s="1">
         <v>99</v>
       </c>
-      <c r="S16" t="s" s="1">
+      <c r="E18" t="s" s="1">
+        <v>30</v>
+      </c>
+      <c r="F18" t="s" s="1">
+        <v>31</v>
+      </c>
+      <c r="G18" t="s" s="1">
+        <v>32</v>
+      </c>
+      <c r="H18" t="s" s="1">
+        <v>30</v>
+      </c>
+      <c r="I18" t="s" s="1">
+        <v>33</v>
+      </c>
+      <c r="J18" t="s" s="1">
         <v>100</v>
       </c>
-      <c r="T16" t="s" s="1">
-        <v>37</v>
-      </c>
-      <c r="Y16" t="s" s="1">
-        <v>62</v>
-      </c>
-      <c r="Z16" t="s" s="1">
-        <v>38</v>
+      <c r="K18" t="s" s="1">
+        <v>31</v>
+      </c>
+      <c r="L18">
+        <v>1</v>
+      </c>
+      <c r="M18">
+        <v>0.5</v>
+      </c>
+      <c r="N18">
+        <v>0.5</v>
+      </c>
+      <c r="O18">
+        <v>0</v>
+      </c>
+      <c r="P18">
+        <v>0</v>
+      </c>
+      <c r="Q18" t="s" s="1">
+        <v>35</v>
+      </c>
+      <c r="R18" t="s" s="1">
+        <v>101</v>
+      </c>
+      <c r="S18" t="s" s="1">
+        <v>102</v>
+      </c>
+      <c r="T18" t="s" s="1">
+        <v>38</v>
+      </c>
+      <c r="Y18" t="s" s="1">
+        <v>100</v>
+      </c>
+      <c r="Z18" t="s" s="1">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="s" s="1">
+        <v>42</v>
+      </c>
+      <c r="B19" t="s" s="1">
+        <v>27</v>
+      </c>
+      <c r="C19" t="s" s="1">
+        <v>28</v>
+      </c>
+      <c r="D19" t="s" s="1">
+        <v>103</v>
+      </c>
+      <c r="E19" t="s" s="1">
+        <v>30</v>
+      </c>
+      <c r="F19" t="s" s="1">
+        <v>31</v>
+      </c>
+      <c r="G19" t="s" s="1">
+        <v>32</v>
+      </c>
+      <c r="H19" t="s" s="1">
+        <v>30</v>
+      </c>
+      <c r="I19" t="s" s="1">
+        <v>33</v>
+      </c>
+      <c r="J19" t="s" s="1">
+        <v>65</v>
+      </c>
+      <c r="K19" t="s" s="1">
+        <v>31</v>
+      </c>
+      <c r="L19">
+        <v>1</v>
+      </c>
+      <c r="M19">
+        <v>0.5</v>
+      </c>
+      <c r="N19">
+        <v>0.5</v>
+      </c>
+      <c r="O19">
+        <v>0</v>
+      </c>
+      <c r="P19">
+        <v>0</v>
+      </c>
+      <c r="Q19" t="s" s="1">
+        <v>35</v>
+      </c>
+      <c r="R19" t="s" s="1">
+        <v>104</v>
+      </c>
+      <c r="S19" t="s" s="1">
+        <v>105</v>
+      </c>
+      <c r="T19" t="s" s="1">
+        <v>38</v>
+      </c>
+      <c r="Y19" t="s" s="1">
+        <v>65</v>
+      </c>
+      <c r="Z19" t="s" s="1">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="s" s="1">
+        <v>106</v>
+      </c>
+      <c r="B20" t="s" s="1">
+        <v>27</v>
+      </c>
+      <c r="C20" t="s" s="1">
+        <v>28</v>
+      </c>
+      <c r="D20" t="s" s="1">
+        <v>107</v>
+      </c>
+      <c r="E20" t="s" s="1">
+        <v>30</v>
+      </c>
+      <c r="F20" t="s" s="1">
+        <v>31</v>
+      </c>
+      <c r="G20" t="s" s="1">
+        <v>32</v>
+      </c>
+      <c r="H20" t="s" s="1">
+        <v>30</v>
+      </c>
+      <c r="I20" t="s" s="1">
+        <v>33</v>
+      </c>
+      <c r="J20" t="s" s="1">
+        <v>34</v>
+      </c>
+      <c r="K20" t="s" s="1">
+        <v>31</v>
+      </c>
+      <c r="L20">
+        <v>1</v>
+      </c>
+      <c r="M20">
+        <v>0.5</v>
+      </c>
+      <c r="N20">
+        <v>0.5</v>
+      </c>
+      <c r="O20">
+        <v>0</v>
+      </c>
+      <c r="P20">
+        <v>0</v>
+      </c>
+      <c r="Q20" t="s" s="1">
+        <v>35</v>
+      </c>
+      <c r="R20" t="s" s="1">
+        <v>108</v>
+      </c>
+      <c r="S20" t="s" s="1">
+        <v>109</v>
+      </c>
+      <c r="T20" t="s" s="1">
+        <v>38</v>
+      </c>
+      <c r="Y20" t="s" s="1">
+        <v>34</v>
+      </c>
+      <c r="Z20" t="s" s="1">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="s" s="1">
+        <v>106</v>
+      </c>
+      <c r="B21" t="s" s="1">
+        <v>27</v>
+      </c>
+      <c r="C21" t="s" s="1">
+        <v>40</v>
+      </c>
+      <c r="D21" t="s" s="1">
+        <v>41</v>
+      </c>
+      <c r="E21" t="s" s="1">
+        <v>30</v>
+      </c>
+      <c r="F21" t="s" s="1">
+        <v>31</v>
+      </c>
+      <c r="G21" t="s" s="1">
+        <v>32</v>
+      </c>
+      <c r="H21" t="s" s="1">
+        <v>30</v>
+      </c>
+      <c r="I21" t="s" s="1">
+        <v>33</v>
+      </c>
+      <c r="J21" t="s" s="1">
+        <v>34</v>
+      </c>
+      <c r="K21" t="s" s="1">
+        <v>31</v>
+      </c>
+      <c r="L21">
+        <v>1</v>
+      </c>
+      <c r="M21">
+        <v>0.5</v>
+      </c>
+      <c r="N21">
+        <v>0.5</v>
+      </c>
+      <c r="O21">
+        <v>0</v>
+      </c>
+      <c r="P21">
+        <v>0</v>
+      </c>
+      <c r="Q21" t="s" s="1">
+        <v>35</v>
+      </c>
+      <c r="R21" t="s" s="1">
+        <v>108</v>
+      </c>
+      <c r="S21" t="s" s="1">
+        <v>110</v>
+      </c>
+      <c r="T21" t="s" s="1">
+        <v>38</v>
+      </c>
+      <c r="Y21" t="s" s="1">
+        <v>34</v>
+      </c>
+      <c r="Z21" t="s" s="1">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="s" s="1">
+        <v>111</v>
+      </c>
+      <c r="B22" t="s" s="1">
+        <v>27</v>
+      </c>
+      <c r="C22" t="s" s="1">
+        <v>28</v>
+      </c>
+      <c r="D22" t="s" s="1">
+        <v>112</v>
+      </c>
+      <c r="E22" t="s" s="1">
+        <v>30</v>
+      </c>
+      <c r="F22" t="s" s="1">
+        <v>31</v>
+      </c>
+      <c r="G22" t="s" s="1">
+        <v>32</v>
+      </c>
+      <c r="H22" t="s" s="1">
+        <v>30</v>
+      </c>
+      <c r="I22" t="s" s="1">
+        <v>33</v>
+      </c>
+      <c r="J22" t="s" s="1">
+        <v>34</v>
+      </c>
+      <c r="K22" t="s" s="1">
+        <v>31</v>
+      </c>
+      <c r="L22">
+        <v>1</v>
+      </c>
+      <c r="M22">
+        <v>0.5</v>
+      </c>
+      <c r="N22">
+        <v>0.5</v>
+      </c>
+      <c r="O22">
+        <v>0</v>
+      </c>
+      <c r="P22">
+        <v>0</v>
+      </c>
+      <c r="Q22" t="s" s="1">
+        <v>35</v>
+      </c>
+      <c r="R22" t="s" s="1">
+        <v>113</v>
+      </c>
+      <c r="S22" t="s" s="1">
+        <v>114</v>
+      </c>
+      <c r="T22" t="s" s="1">
+        <v>38</v>
+      </c>
+      <c r="Y22" t="s" s="1">
+        <v>34</v>
+      </c>
+      <c r="Z22" t="s" s="1">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="s" s="1">
+        <v>111</v>
+      </c>
+      <c r="B23" t="s" s="1">
+        <v>27</v>
+      </c>
+      <c r="C23" t="s" s="1">
+        <v>40</v>
+      </c>
+      <c r="D23" t="s" s="1">
+        <v>115</v>
+      </c>
+      <c r="E23" t="s" s="1">
+        <v>30</v>
+      </c>
+      <c r="F23" t="s" s="1">
+        <v>31</v>
+      </c>
+      <c r="G23" t="s" s="1">
+        <v>32</v>
+      </c>
+      <c r="H23" t="s" s="1">
+        <v>30</v>
+      </c>
+      <c r="I23" t="s" s="1">
+        <v>33</v>
+      </c>
+      <c r="J23" t="s" s="1">
+        <v>34</v>
+      </c>
+      <c r="K23" t="s" s="1">
+        <v>31</v>
+      </c>
+      <c r="L23">
+        <v>1</v>
+      </c>
+      <c r="M23">
+        <v>0.5</v>
+      </c>
+      <c r="N23">
+        <v>0.5</v>
+      </c>
+      <c r="O23">
+        <v>0</v>
+      </c>
+      <c r="P23">
+        <v>0</v>
+      </c>
+      <c r="Q23" t="s" s="1">
+        <v>35</v>
+      </c>
+      <c r="R23" t="s" s="1">
+        <v>116</v>
+      </c>
+      <c r="S23" t="s" s="1">
+        <v>114</v>
+      </c>
+      <c r="T23" t="s" s="1">
+        <v>38</v>
+      </c>
+      <c r="Y23" t="s" s="1">
+        <v>34</v>
+      </c>
+      <c r="Z23" t="s" s="1">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="s" s="1">
+        <v>117</v>
+      </c>
+      <c r="B24" t="s" s="1">
+        <v>27</v>
+      </c>
+      <c r="C24" t="s" s="1">
+        <v>28</v>
+      </c>
+      <c r="D24" t="s" s="1">
+        <v>118</v>
+      </c>
+      <c r="E24" t="s" s="1">
+        <v>30</v>
+      </c>
+      <c r="F24" t="s" s="1">
+        <v>31</v>
+      </c>
+      <c r="G24" t="s" s="1">
+        <v>32</v>
+      </c>
+      <c r="H24" t="s" s="1">
+        <v>30</v>
+      </c>
+      <c r="I24" t="s" s="1">
+        <v>33</v>
+      </c>
+      <c r="J24" t="s" s="1">
+        <v>34</v>
+      </c>
+      <c r="K24" t="s" s="1">
+        <v>31</v>
+      </c>
+      <c r="L24">
+        <v>1</v>
+      </c>
+      <c r="M24">
+        <v>0.5</v>
+      </c>
+      <c r="N24">
+        <v>0.5</v>
+      </c>
+      <c r="O24">
+        <v>0</v>
+      </c>
+      <c r="P24">
+        <v>0</v>
+      </c>
+      <c r="Q24" t="s" s="1">
+        <v>35</v>
+      </c>
+      <c r="R24" t="s" s="1">
+        <v>119</v>
+      </c>
+      <c r="S24" t="s" s="1">
+        <v>120</v>
+      </c>
+      <c r="T24" t="s" s="1">
+        <v>38</v>
+      </c>
+      <c r="Y24" t="s" s="1">
+        <v>34</v>
+      </c>
+      <c r="Z24" t="s" s="1">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="s" s="1">
+        <v>117</v>
+      </c>
+      <c r="B25" t="s" s="1">
+        <v>27</v>
+      </c>
+      <c r="C25" t="s" s="1">
+        <v>40</v>
+      </c>
+      <c r="D25" t="s" s="1">
+        <v>121</v>
+      </c>
+      <c r="E25" t="s" s="1">
+        <v>30</v>
+      </c>
+      <c r="F25" t="s" s="1">
+        <v>31</v>
+      </c>
+      <c r="G25" t="s" s="1">
+        <v>32</v>
+      </c>
+      <c r="H25" t="s" s="1">
+        <v>30</v>
+      </c>
+      <c r="I25" t="s" s="1">
+        <v>33</v>
+      </c>
+      <c r="J25" t="s" s="1">
+        <v>34</v>
+      </c>
+      <c r="K25" t="s" s="1">
+        <v>31</v>
+      </c>
+      <c r="L25">
+        <v>1</v>
+      </c>
+      <c r="M25">
+        <v>0.5</v>
+      </c>
+      <c r="N25">
+        <v>0.5</v>
+      </c>
+      <c r="O25">
+        <v>0</v>
+      </c>
+      <c r="P25">
+        <v>0</v>
+      </c>
+      <c r="Q25" t="s" s="1">
+        <v>35</v>
+      </c>
+      <c r="R25" t="s" s="1">
+        <v>122</v>
+      </c>
+      <c r="S25" t="s" s="1">
+        <v>123</v>
+      </c>
+      <c r="T25" t="s" s="1">
+        <v>38</v>
+      </c>
+      <c r="Y25" t="s" s="1">
+        <v>34</v>
+      </c>
+      <c r="Z25" t="s" s="1">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="s" s="1">
+        <v>124</v>
+      </c>
+      <c r="B26" t="s" s="1">
+        <v>27</v>
+      </c>
+      <c r="C26" t="s" s="1">
+        <v>28</v>
+      </c>
+      <c r="D26" t="s" s="1">
+        <v>125</v>
+      </c>
+      <c r="E26" t="s" s="1">
+        <v>30</v>
+      </c>
+      <c r="F26" t="s" s="1">
+        <v>31</v>
+      </c>
+      <c r="G26" t="s" s="1">
+        <v>32</v>
+      </c>
+      <c r="H26" t="s" s="1">
+        <v>30</v>
+      </c>
+      <c r="I26" t="s" s="1">
+        <v>33</v>
+      </c>
+      <c r="J26" t="s" s="1">
+        <v>34</v>
+      </c>
+      <c r="K26" t="s" s="1">
+        <v>31</v>
+      </c>
+      <c r="L26">
+        <v>1</v>
+      </c>
+      <c r="M26">
+        <v>0.5</v>
+      </c>
+      <c r="N26">
+        <v>0.5</v>
+      </c>
+      <c r="O26">
+        <v>0</v>
+      </c>
+      <c r="P26">
+        <v>0</v>
+      </c>
+      <c r="Q26" t="s" s="1">
+        <v>35</v>
+      </c>
+      <c r="R26" t="s" s="1">
+        <v>126</v>
+      </c>
+      <c r="S26" t="s" s="1">
+        <v>127</v>
+      </c>
+      <c r="T26" t="s" s="1">
+        <v>38</v>
+      </c>
+      <c r="Y26" t="s" s="1">
+        <v>34</v>
+      </c>
+      <c r="Z26" t="s" s="1">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="s" s="1">
+        <v>124</v>
+      </c>
+      <c r="B27" t="s" s="1">
+        <v>27</v>
+      </c>
+      <c r="C27" t="s" s="1">
+        <v>128</v>
+      </c>
+      <c r="D27" t="s" s="1">
+        <v>129</v>
+      </c>
+      <c r="E27" t="s" s="1">
+        <v>30</v>
+      </c>
+      <c r="F27" t="s" s="1">
+        <v>31</v>
+      </c>
+      <c r="G27" t="s" s="1">
+        <v>32</v>
+      </c>
+      <c r="H27" t="s" s="1">
+        <v>30</v>
+      </c>
+      <c r="I27" t="s" s="1">
+        <v>33</v>
+      </c>
+      <c r="J27" t="s" s="1">
+        <v>34</v>
+      </c>
+      <c r="K27" t="s" s="1">
+        <v>31</v>
+      </c>
+      <c r="L27">
+        <v>1</v>
+      </c>
+      <c r="M27">
+        <v>0.5</v>
+      </c>
+      <c r="N27">
+        <v>0.5</v>
+      </c>
+      <c r="O27">
+        <v>0</v>
+      </c>
+      <c r="P27">
+        <v>0</v>
+      </c>
+      <c r="Q27" t="s" s="1">
+        <v>35</v>
+      </c>
+      <c r="R27" t="s" s="1">
+        <v>126</v>
+      </c>
+      <c r="S27" t="s" s="1">
+        <v>127</v>
+      </c>
+      <c r="T27" t="s" s="1">
+        <v>38</v>
+      </c>
+      <c r="Y27" t="s" s="1">
+        <v>34</v>
+      </c>
+      <c r="Z27" t="s" s="1">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="s" s="1">
+        <v>130</v>
+      </c>
+      <c r="B28" t="s" s="1">
+        <v>27</v>
+      </c>
+      <c r="C28" t="s" s="1">
+        <v>40</v>
+      </c>
+      <c r="D28" t="s" s="1">
+        <v>131</v>
+      </c>
+      <c r="E28" t="s" s="1">
+        <v>30</v>
+      </c>
+      <c r="F28" t="s" s="1">
+        <v>31</v>
+      </c>
+      <c r="G28" t="s" s="1">
+        <v>32</v>
+      </c>
+      <c r="H28" t="s" s="1">
+        <v>30</v>
+      </c>
+      <c r="I28" t="s" s="1">
+        <v>33</v>
+      </c>
+      <c r="J28" t="s" s="1">
+        <v>34</v>
+      </c>
+      <c r="K28" t="s" s="1">
+        <v>31</v>
+      </c>
+      <c r="L28">
+        <v>1</v>
+      </c>
+      <c r="M28">
+        <v>0.5</v>
+      </c>
+      <c r="N28">
+        <v>0.5</v>
+      </c>
+      <c r="O28">
+        <v>0</v>
+      </c>
+      <c r="P28">
+        <v>0</v>
+      </c>
+      <c r="Q28" t="s" s="1">
+        <v>35</v>
+      </c>
+      <c r="R28" t="s" s="1">
+        <v>132</v>
+      </c>
+      <c r="S28" t="s" s="1">
+        <v>133</v>
+      </c>
+      <c r="T28" t="s" s="1">
+        <v>38</v>
+      </c>
+      <c r="Y28" t="s" s="1">
+        <v>34</v>
+      </c>
+      <c r="Z28" t="s" s="1">
+        <v>39</v>
       </c>
     </row>
   </sheetData>

</xml_diff>